<commit_message>
Richtiges Gantt Diagram hinzugefügt :)
</commit_message>
<xml_diff>
--- a/Gantt/Einfaches Gantt-Diagramm1.xlsx
+++ b/Gantt/Einfaches Gantt-Diagramm1.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{01165936-CD09-43E3-953F-51C243D9AE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6287BEF5-98BB-4D33-9DBA-F36DD159B441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1335" yWindow="2430" windowWidth="18675" windowHeight="9308" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projektplan" sheetId="11" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <definedName name="task_progress" localSheetId="0">Projektplan!$D1</definedName>
     <definedName name="task_start" localSheetId="0">Projektplan!$E1</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -32,6 +32,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="73">
   <si>
     <t>Erstellen Sie auf diesem Arbeitsblatt einen Projektplan.
 Geben Sie den Titel dieses Projekts in Zelle B1 ein. 
@@ -47,10 +49,22 @@
 Navigieren Sie weiterhin in Spalte A abwärts, um weitere Anweisungen zu hören.</t>
   </si>
   <si>
+    <t>Vogel Lexikon Webseite</t>
+  </si>
+  <si>
     <t>Geben Sie den Firmennamen in Zelle B2 ein.</t>
   </si>
   <si>
+    <t>Firmenname</t>
+  </si>
+  <si>
+    <t>Fafejato</t>
+  </si>
+  <si>
     <t>Geben Sie den Namen des Projektleiters in Zelle B3 ein. Geben Sie das Startdatum für das Projekt in Zelle E3 ein. Start des Projekts: Die Bezeichnung steht in Zelle C3.</t>
+  </si>
+  <si>
+    <t>Projektanfang:</t>
   </si>
   <si>
     <t>Die Anzeigewoche in Zelle E4 stellt die Anfangswoche dar, die im Projektplan in Zelle I4 angezeigt werden soll. Das Startdatum des Projekts wird als Woche 1 betrachtet. Um die Anzeigewoche zu ändern, geben Sie einfach eine neue Wochennummer in Zelle E4 ein.
@@ -59,6 +73,9 @@
 Anzeigewoche: Die Bezeichnung steht in Zelle C4.</t>
   </si>
   <si>
+    <t>Anzeigewoche:</t>
+  </si>
+  <si>
     <t>Die Zellen I5 bis BL5 enthalten die Tagesnummer der Woche für die im Zellenblock oberhalb der einzelnen Datumszellen angezeigten Woche und werden automatisch berechnet.
 Ändern Sie diese Zellen nicht.
 Das heutige Datum ist rot (Hex #AD3815) hervorgehoben, vom aktuellen Datum in Zeile 5 die gesamte Datumsspalte hindurch bis zum Ende des Projektplans.</t>
@@ -68,6 +85,25 @@
 Navigieren Sie von B6 bis BL6, um sich die Inhalte vorsprechen zu lassen. Der erste Buchstabe jedes Tags der Woche für das Datum oberhalb der Überschrift, beginnend in Zelle I6 und fortlaufend bis Zelle BL6.
 Alle Projektzeitachsendiagramme werden automatisch basierend auf den eingegebenen Start- und Enddaten mithilfe von bedingten Formaten generiert.
 Ändern Sie die Inhalte in den Zellen in Spalten nach Spalte I beginnend mit Zelle I7 nicht.</t>
+  </si>
+  <si>
+    <t>AUFGABE</t>
+  </si>
+  <si>
+    <t>ZUGEWIESEN
+AN</t>
+  </si>
+  <si>
+    <t>FORTSCHRITT</t>
+  </si>
+  <si>
+    <t>START</t>
+  </si>
+  <si>
+    <t>ENDE</t>
+  </si>
+  <si>
+    <t>TAGE</t>
   </si>
   <si>
     <t xml:space="preserve">Löschen Sie diese Zeile nicht. Diese Zeile ist ausgeblendet, um eine Formel zu schützen, die zum Hervorheben des aktuellen Tags im Projektzeitplan verwendet wird. </t>
@@ -82,6 +118,9 @@
 Um die Phase zu löschen und nur mit Aufgaben zu arbeiten, löschen Sie einfach diese Zeile.</t>
   </si>
   <si>
+    <t>Phase 1 Mock Up</t>
+  </si>
+  <si>
     <t xml:space="preserve">Zelle B9 enthält die Beispielaufgabe „Aufgabe 1“. 
 Geben Sie einen neuen Aufgabennamen in Zelle B9 ein.
 Geben Sie in Zelle C9 eine Person ein, der die Aufgabe zugewiesen werden soll.
@@ -91,10 +130,37 @@
 Von Zelle I9 bis Zelle BL9 wird eine Statusleiste mit einer entsprechenden Schattierung für die eingegebenen Datumsangaben in Blöcken angezeigt. </t>
   </si>
   <si>
+    <t>Projektvorstellung, Motivation, Intention</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>In den Zeilen 10 bis 13 wird das Muster aus Zeile 9 wiederholt. 
 Wiederholen Sie die Anweisungen aus Zelle A9 für alle Aufgabenzeilen auf diesem Arbeitsblatt. Überschreiben Sie alle Beispieldaten.
 Ein Beispiel für eine andere Phase beginnt in Zelle A14. 
 Setzen Sie die Eingabe von Aufgaben in den Zellen A10 bis A13 fort, oder wechseln Sie zu Zelle A14, um weitere Informationen zu erhalten.</t>
+  </si>
+  <si>
+    <t>Zieldefinition</t>
+  </si>
+  <si>
+    <t>Abschätzung des Projektumfangs</t>
+  </si>
+  <si>
+    <t>Organisationsplanung</t>
+  </si>
+  <si>
+    <t>Mock Up/Zoachning</t>
+  </si>
+  <si>
+    <t>Thorben, Team</t>
+  </si>
+  <si>
+    <t>Powerpoint erstellen</t>
+  </si>
+  <si>
+    <t>Team, Fabian</t>
   </si>
   <si>
     <t>Die Zelle rechts enthält den Beispieltitel „Phase 2“. 
@@ -107,7 +173,73 @@
 Wiederholen Sie bei Bedarf die Anweisungen aus den Zellen A8 und A9.</t>
   </si>
   <si>
+    <t>Phase 2 Html Prototyp</t>
+  </si>
+  <si>
+    <t>Landing Page/Suche</t>
+  </si>
+  <si>
+    <t>Browseseite</t>
+  </si>
+  <si>
+    <t>Detailseite</t>
+  </si>
+  <si>
+    <t>Felix, Fabian</t>
+  </si>
+  <si>
+    <t>Login/User</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Forum</t>
+  </si>
+  <si>
     <t>Titelblock für Beispielphase</t>
+  </si>
+  <si>
+    <t>Phase 3 Dynamischer Prototyp</t>
+  </si>
+  <si>
+    <t>Backend implementieren</t>
+  </si>
+  <si>
+    <t>Thorben</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontendpages dynamisch machen </t>
+  </si>
+  <si>
+    <t>Formulare erzeugen</t>
+  </si>
+  <si>
+    <t>Zusammenpacken  der einzelnen Seiten</t>
+  </si>
+  <si>
+    <t>Testen, Testen, Testen</t>
+  </si>
+  <si>
+    <t>Phase 4 Final Release</t>
+  </si>
+  <si>
+    <t>Aufgabe 1</t>
+  </si>
+  <si>
+    <t>Datum</t>
+  </si>
+  <si>
+    <t>Aufgabe 2</t>
+  </si>
+  <si>
+    <t>Aufgabe 3</t>
+  </si>
+  <si>
+    <t>Aufgabe 4</t>
+  </si>
+  <si>
+    <t>Aufgabe 5</t>
   </si>
   <si>
     <t>Dies ist eine leere Zeile.</t>
@@ -117,71 +249,7 @@
 Fügen Sie ÜBER dieser Zeile neue Zeilen ein, um mit der Erstellung Ihres Projektplans fortzufahren.</t>
   </si>
   <si>
-    <t>Firmenname</t>
-  </si>
-  <si>
-    <t>Projektleiter</t>
-  </si>
-  <si>
-    <t>AUFGABE</t>
-  </si>
-  <si>
-    <t>Phase 1 Titel</t>
-  </si>
-  <si>
-    <t>Aufgabe 1</t>
-  </si>
-  <si>
-    <t>Aufgabe 2</t>
-  </si>
-  <si>
-    <t>Aufgabe 3</t>
-  </si>
-  <si>
-    <t>Aufgabe 4</t>
-  </si>
-  <si>
-    <t>Aufgabe 5</t>
-  </si>
-  <si>
-    <t>Phase 2 Titel</t>
-  </si>
-  <si>
-    <t>Phase 3 Titel</t>
-  </si>
-  <si>
-    <t>Phase 4 Titel</t>
-  </si>
-  <si>
     <t>Neue Zeilen ÜBER dieser einfügen</t>
-  </si>
-  <si>
-    <t>Projektanfang:</t>
-  </si>
-  <si>
-    <t>Anzeigewoche:</t>
-  </si>
-  <si>
-    <t>ZUGEWIESEN
-AN</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>FORTSCHRITT</t>
-  </si>
-  <si>
-    <t>START</t>
-  </si>
-  <si>
-    <t>Datum</t>
-  </si>
-  <si>
-    <t>ENDE</t>
-  </si>
-  <si>
-    <t>TAGE</t>
   </si>
   <si>
     <t>EINFACHES GANTT-DIAGRAMM von Vertex42.com</t>
@@ -232,12 +300,6 @@
   </si>
   <si>
     <t>Unternehmen werden bei Rechnungen, Arbeitszeittabellen, Bestandstrackern, Geschäftsberichten und Vorlagen für die Projektplanung fündig. Lehrer und Schüler finden Ressourcen wie Stundenpläne, Klassenbücher und Teilnahmebögen. Organisieren Sie Ihr Familienleben mit Speiseplänen, Checklisten und Übungsprotokollen. Jede Vorlage wurde gründlich recherchiert, verfeinert und im Lauf der Zeit anhand des Feedbacks von Tausenden von Benutzern verbessert.</t>
-  </si>
-  <si>
-    <t>Vogel Lexikon Webseite</t>
-  </si>
-  <si>
-    <t>Fafejato</t>
   </si>
 </sst>
 </file>
@@ -1194,9 +1256,6 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="11" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="11" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="2" xfId="11" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1217,12 +1276,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="11">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="12" applyFill="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="12" applyFill="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="11" borderId="2" xfId="12" applyFill="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
@@ -1295,23 +1348,32 @@
     <xf numFmtId="170" fontId="11" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="12" applyFont="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="11" applyFont="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="12" applyFont="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="3" xfId="9">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8">
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1">
       <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="9" fillId="0" borderId="3" xfId="9">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="54">
@@ -1370,7 +1432,7 @@
     <cellStyle name="zAusgeblText" xfId="3" xr:uid="{26E66EE6-E33F-4D77-BAE4-0FB4F5BBF673}"/>
     <cellStyle name="Zelle überprüfen" xfId="25" builtinId="23" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="13">
     <dxf>
       <fill>
         <patternFill>
@@ -1388,6 +1450,17 @@
           <bgColor theme="0" tint="-0.34998626667073579"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+      </border>
     </dxf>
     <dxf>
       <border>
@@ -1497,15 +1570,15 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Aufgabenliste" pivot="0" count="9" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="11"/>
-      <tableStyleElement type="headerRow" dxfId="10"/>
-      <tableStyleElement type="totalRow" dxfId="9"/>
-      <tableStyleElement type="firstColumn" dxfId="8"/>
-      <tableStyleElement type="lastColumn" dxfId="7"/>
-      <tableStyleElement type="firstRowStripe" dxfId="6"/>
-      <tableStyleElement type="secondRowStripe" dxfId="5"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="4"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="3"/>
+      <tableStyleElement type="wholeTable" dxfId="12"/>
+      <tableStyleElement type="headerRow" dxfId="11"/>
+      <tableStyleElement type="totalRow" dxfId="10"/>
+      <tableStyleElement type="firstColumn" dxfId="9"/>
+      <tableStyleElement type="lastColumn" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="secondRowStripe" dxfId="6"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="5"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="4"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -1652,6 +1725,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1920,12 +1997,12 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BL36"/>
+  <dimension ref="A1:BL37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.73046875" style="45" customWidth="1"/>
-    <col min="2" max="2" width="19.86328125" customWidth="1"/>
-    <col min="3" max="3" width="30.73046875" customWidth="1"/>
+    <col min="2" max="2" width="37.1328125" customWidth="1"/>
+    <col min="3" max="3" width="23.1328125" customWidth="1"/>
     <col min="4" max="4" width="10.73046875" customWidth="1"/>
     <col min="5" max="5" width="10.3984375" style="5" customWidth="1"/>
     <col min="6" max="6" width="10.3984375" customWidth="1"/>
@@ -1940,397 +2017,391 @@
         <v>0</v>
       </c>
       <c r="B1" s="49" t="s">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="2"/>
       <c r="E1" s="4"/>
       <c r="F1" s="34"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="67" t="s">
-        <v>36</v>
-      </c>
+      <c r="I1" s="64"/>
     </row>
     <row r="2" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="45" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" s="50" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
-      </c>
-      <c r="I2" s="68" t="s">
-        <v>37</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="I2" s="65"/>
     </row>
     <row r="3" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="45" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="51" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="88" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="89"/>
-      <c r="E3" s="93">
+        <v>5</v>
+      </c>
+      <c r="B3" s="51"/>
+      <c r="C3" s="92" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="93"/>
+      <c r="E3" s="91">
         <f ca="1">TODAY()</f>
         <v>46108</v>
       </c>
-      <c r="F3" s="93"/>
+      <c r="F3" s="91"/>
     </row>
     <row r="4" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="46" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="88" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="89"/>
+        <v>7</v>
+      </c>
+      <c r="C4" s="92" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="93"/>
       <c r="E4" s="7">
         <v>1</v>
       </c>
-      <c r="I4" s="90">
+      <c r="I4" s="88">
         <f ca="1">I5</f>
         <v>46104</v>
       </c>
-      <c r="J4" s="91"/>
-      <c r="K4" s="91"/>
-      <c r="L4" s="91"/>
-      <c r="M4" s="91"/>
-      <c r="N4" s="91"/>
-      <c r="O4" s="92"/>
-      <c r="P4" s="90">
+      <c r="J4" s="89"/>
+      <c r="K4" s="89"/>
+      <c r="L4" s="89"/>
+      <c r="M4" s="89"/>
+      <c r="N4" s="89"/>
+      <c r="O4" s="90"/>
+      <c r="P4" s="88">
         <f ca="1">P5</f>
         <v>46111</v>
       </c>
-      <c r="Q4" s="91"/>
-      <c r="R4" s="91"/>
-      <c r="S4" s="91"/>
-      <c r="T4" s="91"/>
-      <c r="U4" s="91"/>
-      <c r="V4" s="92"/>
-      <c r="W4" s="90">
+      <c r="Q4" s="89"/>
+      <c r="R4" s="89"/>
+      <c r="S4" s="89"/>
+      <c r="T4" s="89"/>
+      <c r="U4" s="89"/>
+      <c r="V4" s="90"/>
+      <c r="W4" s="88">
         <f ca="1">W5</f>
         <v>46118</v>
       </c>
-      <c r="X4" s="91"/>
-      <c r="Y4" s="91"/>
-      <c r="Z4" s="91"/>
-      <c r="AA4" s="91"/>
-      <c r="AB4" s="91"/>
-      <c r="AC4" s="92"/>
-      <c r="AD4" s="90">
+      <c r="X4" s="89"/>
+      <c r="Y4" s="89"/>
+      <c r="Z4" s="89"/>
+      <c r="AA4" s="89"/>
+      <c r="AB4" s="89"/>
+      <c r="AC4" s="90"/>
+      <c r="AD4" s="88">
         <f ca="1">AD5</f>
         <v>46125</v>
       </c>
-      <c r="AE4" s="91"/>
-      <c r="AF4" s="91"/>
-      <c r="AG4" s="91"/>
-      <c r="AH4" s="91"/>
-      <c r="AI4" s="91"/>
-      <c r="AJ4" s="92"/>
-      <c r="AK4" s="90">
+      <c r="AE4" s="89"/>
+      <c r="AF4" s="89"/>
+      <c r="AG4" s="89"/>
+      <c r="AH4" s="89"/>
+      <c r="AI4" s="89"/>
+      <c r="AJ4" s="90"/>
+      <c r="AK4" s="88">
         <f ca="1">AK5</f>
         <v>46132</v>
       </c>
-      <c r="AL4" s="91"/>
-      <c r="AM4" s="91"/>
-      <c r="AN4" s="91"/>
-      <c r="AO4" s="91"/>
-      <c r="AP4" s="91"/>
-      <c r="AQ4" s="92"/>
-      <c r="AR4" s="90">
+      <c r="AL4" s="89"/>
+      <c r="AM4" s="89"/>
+      <c r="AN4" s="89"/>
+      <c r="AO4" s="89"/>
+      <c r="AP4" s="89"/>
+      <c r="AQ4" s="90"/>
+      <c r="AR4" s="88">
         <f ca="1">AR5</f>
         <v>46139</v>
       </c>
-      <c r="AS4" s="91"/>
-      <c r="AT4" s="91"/>
-      <c r="AU4" s="91"/>
-      <c r="AV4" s="91"/>
-      <c r="AW4" s="91"/>
-      <c r="AX4" s="92"/>
-      <c r="AY4" s="90">
+      <c r="AS4" s="89"/>
+      <c r="AT4" s="89"/>
+      <c r="AU4" s="89"/>
+      <c r="AV4" s="89"/>
+      <c r="AW4" s="89"/>
+      <c r="AX4" s="90"/>
+      <c r="AY4" s="88">
         <f ca="1">AY5</f>
         <v>46146</v>
       </c>
-      <c r="AZ4" s="91"/>
-      <c r="BA4" s="91"/>
-      <c r="BB4" s="91"/>
-      <c r="BC4" s="91"/>
-      <c r="BD4" s="91"/>
-      <c r="BE4" s="92"/>
-      <c r="BF4" s="90">
+      <c r="AZ4" s="89"/>
+      <c r="BA4" s="89"/>
+      <c r="BB4" s="89"/>
+      <c r="BC4" s="89"/>
+      <c r="BD4" s="89"/>
+      <c r="BE4" s="90"/>
+      <c r="BF4" s="88">
         <f ca="1">BF5</f>
         <v>46153</v>
       </c>
-      <c r="BG4" s="91"/>
-      <c r="BH4" s="91"/>
-      <c r="BI4" s="91"/>
-      <c r="BJ4" s="91"/>
-      <c r="BK4" s="91"/>
-      <c r="BL4" s="92"/>
+      <c r="BG4" s="89"/>
+      <c r="BH4" s="89"/>
+      <c r="BI4" s="89"/>
+      <c r="BJ4" s="89"/>
+      <c r="BK4" s="89"/>
+      <c r="BL4" s="90"/>
     </row>
     <row r="5" spans="1:64" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="46" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="66"/>
-      <c r="C5" s="66"/>
-      <c r="D5" s="66"/>
-      <c r="E5" s="66"/>
-      <c r="F5" s="66"/>
-      <c r="G5" s="66"/>
-      <c r="I5" s="85">
+        <v>9</v>
+      </c>
+      <c r="B5" s="63"/>
+      <c r="C5" s="63"/>
+      <c r="D5" s="63"/>
+      <c r="E5" s="63"/>
+      <c r="F5" s="63"/>
+      <c r="G5" s="63"/>
+      <c r="I5" s="82">
         <f ca="1">Projektanfang-WEEKDAY(Projektanfang,1)+2+7*(Anzeigewoche-1)</f>
         <v>46104</v>
       </c>
-      <c r="J5" s="86">
+      <c r="J5" s="83">
         <f ca="1">I5+1</f>
         <v>46105</v>
       </c>
-      <c r="K5" s="86">
+      <c r="K5" s="83">
         <f t="shared" ref="K5:AX5" ca="1" si="0">J5+1</f>
         <v>46106</v>
       </c>
-      <c r="L5" s="86">
+      <c r="L5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46107</v>
       </c>
-      <c r="M5" s="86">
+      <c r="M5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46108</v>
       </c>
-      <c r="N5" s="86">
+      <c r="N5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46109</v>
       </c>
-      <c r="O5" s="87">
+      <c r="O5" s="84">
         <f t="shared" ca="1" si="0"/>
         <v>46110</v>
       </c>
-      <c r="P5" s="85">
+      <c r="P5" s="82">
         <f ca="1">O5+1</f>
         <v>46111</v>
       </c>
-      <c r="Q5" s="86">
+      <c r="Q5" s="83">
         <f ca="1">P5+1</f>
         <v>46112</v>
       </c>
-      <c r="R5" s="86">
+      <c r="R5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46113</v>
       </c>
-      <c r="S5" s="86">
+      <c r="S5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46114</v>
       </c>
-      <c r="T5" s="86">
+      <c r="T5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46115</v>
       </c>
-      <c r="U5" s="86">
+      <c r="U5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46116</v>
       </c>
-      <c r="V5" s="87">
+      <c r="V5" s="84">
         <f t="shared" ca="1" si="0"/>
         <v>46117</v>
       </c>
-      <c r="W5" s="85">
+      <c r="W5" s="82">
         <f ca="1">V5+1</f>
         <v>46118</v>
       </c>
-      <c r="X5" s="86">
+      <c r="X5" s="83">
         <f ca="1">W5+1</f>
         <v>46119</v>
       </c>
-      <c r="Y5" s="86">
+      <c r="Y5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46120</v>
       </c>
-      <c r="Z5" s="86">
+      <c r="Z5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46121</v>
       </c>
-      <c r="AA5" s="86">
+      <c r="AA5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46122</v>
       </c>
-      <c r="AB5" s="86">
+      <c r="AB5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46123</v>
       </c>
-      <c r="AC5" s="87">
+      <c r="AC5" s="84">
         <f t="shared" ca="1" si="0"/>
         <v>46124</v>
       </c>
-      <c r="AD5" s="85">
+      <c r="AD5" s="82">
         <f ca="1">AC5+1</f>
         <v>46125</v>
       </c>
-      <c r="AE5" s="86">
+      <c r="AE5" s="83">
         <f ca="1">AD5+1</f>
         <v>46126</v>
       </c>
-      <c r="AF5" s="86">
+      <c r="AF5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46127</v>
       </c>
-      <c r="AG5" s="86">
+      <c r="AG5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46128</v>
       </c>
-      <c r="AH5" s="86">
+      <c r="AH5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46129</v>
       </c>
-      <c r="AI5" s="86">
+      <c r="AI5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46130</v>
       </c>
-      <c r="AJ5" s="87">
+      <c r="AJ5" s="84">
         <f t="shared" ca="1" si="0"/>
         <v>46131</v>
       </c>
-      <c r="AK5" s="85">
+      <c r="AK5" s="82">
         <f ca="1">AJ5+1</f>
         <v>46132</v>
       </c>
-      <c r="AL5" s="86">
+      <c r="AL5" s="83">
         <f ca="1">AK5+1</f>
         <v>46133</v>
       </c>
-      <c r="AM5" s="86">
+      <c r="AM5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46134</v>
       </c>
-      <c r="AN5" s="86">
+      <c r="AN5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46135</v>
       </c>
-      <c r="AO5" s="86">
+      <c r="AO5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46136</v>
       </c>
-      <c r="AP5" s="86">
+      <c r="AP5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46137</v>
       </c>
-      <c r="AQ5" s="87">
+      <c r="AQ5" s="84">
         <f t="shared" ca="1" si="0"/>
         <v>46138</v>
       </c>
-      <c r="AR5" s="85">
+      <c r="AR5" s="82">
         <f ca="1">AQ5+1</f>
         <v>46139</v>
       </c>
-      <c r="AS5" s="86">
+      <c r="AS5" s="83">
         <f ca="1">AR5+1</f>
         <v>46140</v>
       </c>
-      <c r="AT5" s="86">
+      <c r="AT5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46141</v>
       </c>
-      <c r="AU5" s="86">
+      <c r="AU5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46142</v>
       </c>
-      <c r="AV5" s="86">
+      <c r="AV5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46143</v>
       </c>
-      <c r="AW5" s="86">
+      <c r="AW5" s="83">
         <f t="shared" ca="1" si="0"/>
         <v>46144</v>
       </c>
-      <c r="AX5" s="87">
+      <c r="AX5" s="84">
         <f t="shared" ca="1" si="0"/>
         <v>46145</v>
       </c>
-      <c r="AY5" s="85">
+      <c r="AY5" s="82">
         <f ca="1">AX5+1</f>
         <v>46146</v>
       </c>
-      <c r="AZ5" s="86">
+      <c r="AZ5" s="83">
         <f ca="1">AY5+1</f>
         <v>46147</v>
       </c>
-      <c r="BA5" s="86">
+      <c r="BA5" s="83">
         <f t="shared" ref="BA5:BE5" ca="1" si="1">AZ5+1</f>
         <v>46148</v>
       </c>
-      <c r="BB5" s="86">
+      <c r="BB5" s="83">
         <f t="shared" ca="1" si="1"/>
         <v>46149</v>
       </c>
-      <c r="BC5" s="86">
+      <c r="BC5" s="83">
         <f t="shared" ca="1" si="1"/>
         <v>46150</v>
       </c>
-      <c r="BD5" s="86">
+      <c r="BD5" s="83">
         <f t="shared" ca="1" si="1"/>
         <v>46151</v>
       </c>
-      <c r="BE5" s="87">
+      <c r="BE5" s="84">
         <f t="shared" ca="1" si="1"/>
         <v>46152</v>
       </c>
-      <c r="BF5" s="85">
+      <c r="BF5" s="82">
         <f ca="1">BE5+1</f>
         <v>46153</v>
       </c>
-      <c r="BG5" s="86">
+      <c r="BG5" s="83">
         <f ca="1">BF5+1</f>
         <v>46154</v>
       </c>
-      <c r="BH5" s="86">
+      <c r="BH5" s="83">
         <f t="shared" ref="BH5:BL5" ca="1" si="2">BG5+1</f>
         <v>46155</v>
       </c>
-      <c r="BI5" s="86">
+      <c r="BI5" s="83">
         <f t="shared" ca="1" si="2"/>
         <v>46156</v>
       </c>
-      <c r="BJ5" s="86">
+      <c r="BJ5" s="83">
         <f t="shared" ca="1" si="2"/>
         <v>46157</v>
       </c>
-      <c r="BK5" s="86">
+      <c r="BK5" s="83">
         <f t="shared" ca="1" si="2"/>
         <v>46158</v>
       </c>
-      <c r="BL5" s="87">
+      <c r="BL5" s="84">
         <f t="shared" ca="1" si="2"/>
         <v>46159</v>
       </c>
     </row>
     <row r="6" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="46" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="G6" s="9"/>
       <c r="H6" s="9" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="I6" s="10" t="str">
         <f t="shared" ref="I6:AN6" ca="1" si="3">LEFT(TEXT(I5,"TTT"),1)</f>
@@ -2461,7 +2532,7 @@
         <v>D</v>
       </c>
       <c r="AO6" s="10" t="str">
-        <f t="shared" ref="AO6:BT6" ca="1" si="4">LEFT(TEXT(AO5,"TTT"),1)</f>
+        <f t="shared" ref="AO6:BL6" ca="1" si="4">LEFT(TEXT(AO5,"TTT"),1)</f>
         <v>F</v>
       </c>
       <c r="AP6" s="10" t="str">
@@ -2559,7 +2630,7 @@
     </row>
     <row r="7" spans="1:64" ht="39.4" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A7" s="45" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="C7" s="48"/>
       <c r="E7"/>
@@ -2626,18 +2697,18 @@
     </row>
     <row r="8" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A8" s="46" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C8" s="52"/>
       <c r="D8" s="16"/>
-      <c r="E8" s="70"/>
-      <c r="F8" s="71"/>
+      <c r="E8" s="67"/>
+      <c r="F8" s="68"/>
       <c r="G8" s="14"/>
       <c r="H8" s="14" t="str">
-        <f t="shared" ref="H8:H33" si="5">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f t="shared" ref="H8:H34" si="5">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="I8" s="31"/>
@@ -2699,29 +2770,28 @@
     </row>
     <row r="9" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A9" s="46" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="61" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="53" t="s">
-        <v>30</v>
+        <v>20</v>
+      </c>
+      <c r="B9" s="85" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="86" t="s">
+        <v>22</v>
       </c>
       <c r="D9" s="17">
-        <v>0.5</v>
-      </c>
-      <c r="E9" s="72">
+        <v>1</v>
+      </c>
+      <c r="E9" s="69">
         <f ca="1">Projektanfang</f>
         <v>46108</v>
       </c>
-      <c r="F9" s="72">
-        <f ca="1">E9+3</f>
-        <v>46111</v>
+      <c r="F9" s="69">
+        <v>46108</v>
       </c>
       <c r="G9" s="14"/>
       <c r="H9" s="14">
         <f t="shared" ca="1" si="5"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I9" s="31"/>
       <c r="J9" s="31"/>
@@ -2733,7 +2803,6 @@
       <c r="P9" s="31"/>
       <c r="Q9" s="31"/>
       <c r="R9" s="31"/>
-      <c r="S9" s="31"/>
       <c r="T9" s="31"/>
       <c r="U9" s="31"/>
       <c r="V9" s="31"/>
@@ -2782,27 +2851,28 @@
     </row>
     <row r="10" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A10" s="46" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="61" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="53"/>
+        <v>23</v>
+      </c>
+      <c r="B10" s="85" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="86" t="s">
+        <v>22</v>
+      </c>
       <c r="D10" s="17">
-        <v>0.6</v>
-      </c>
-      <c r="E10" s="72">
-        <f ca="1">F9</f>
-        <v>46111</v>
-      </c>
-      <c r="F10" s="72">
-        <f ca="1">E10+2</f>
-        <v>46113</v>
+        <v>1</v>
+      </c>
+      <c r="E10" s="69">
+        <f>F9</f>
+        <v>46108</v>
+      </c>
+      <c r="F10" s="69">
+        <v>46108</v>
       </c>
       <c r="G10" s="14"/>
       <c r="H10" s="14">
-        <f t="shared" ca="1" si="5"/>
-        <v>3</v>
+        <f t="shared" si="5"/>
+        <v>1</v>
       </c>
       <c r="I10" s="31"/>
       <c r="J10" s="31"/>
@@ -2863,25 +2933,26 @@
     </row>
     <row r="11" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A11" s="45"/>
-      <c r="B11" s="61" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="53"/>
+      <c r="B11" s="85" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="86" t="s">
+        <v>22</v>
+      </c>
       <c r="D11" s="17">
-        <v>0.5</v>
-      </c>
-      <c r="E11" s="72">
-        <f ca="1">F10</f>
-        <v>46113</v>
-      </c>
-      <c r="F11" s="72">
-        <f ca="1">E11+4</f>
-        <v>46117</v>
+        <v>0.9</v>
+      </c>
+      <c r="E11" s="69">
+        <f>F10</f>
+        <v>46108</v>
+      </c>
+      <c r="F11" s="69">
+        <v>46108</v>
       </c>
       <c r="G11" s="14"/>
       <c r="H11" s="14">
-        <f t="shared" ca="1" si="5"/>
-        <v>5</v>
+        <f t="shared" si="5"/>
+        <v>1</v>
       </c>
       <c r="I11" s="31"/>
       <c r="J11" s="31"/>
@@ -2940,27 +3011,28 @@
       <c r="BK11" s="31"/>
       <c r="BL11" s="31"/>
     </row>
-    <row r="12" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="45"/>
-      <c r="B12" s="61" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="53"/>
+      <c r="B12" s="85" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="86" t="s">
+        <v>22</v>
+      </c>
       <c r="D12" s="17">
         <v>0.25</v>
       </c>
-      <c r="E12" s="72">
-        <f ca="1">F11</f>
-        <v>46117</v>
-      </c>
-      <c r="F12" s="72">
-        <f ca="1">E12+5</f>
-        <v>46122</v>
+      <c r="E12" s="69">
+        <f>F11</f>
+        <v>46108</v>
+      </c>
+      <c r="F12" s="69">
+        <v>46108</v>
       </c>
       <c r="G12" s="14"/>
       <c r="H12" s="14">
-        <f t="shared" ca="1" si="5"/>
-        <v>6</v>
+        <f t="shared" si="5"/>
+        <v>1</v>
       </c>
       <c r="I12" s="31"/>
       <c r="J12" s="31"/>
@@ -3019,26 +3091,27 @@
       <c r="BK12" s="31"/>
       <c r="BL12" s="31"/>
     </row>
-    <row r="13" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="13" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="45"/>
-      <c r="B13" s="61" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" s="53"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="72">
-        <f ca="1">E10+1</f>
-        <v>46112</v>
-      </c>
-      <c r="F13" s="72">
+      <c r="B13" s="85" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="86" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13" s="17">
+        <v>0.1</v>
+      </c>
+      <c r="E13" s="69">
+        <f ca="1">E9+1</f>
+        <v>46109</v>
+      </c>
+      <c r="F13" s="69">
         <f ca="1">E13+2</f>
-        <v>46114</v>
+        <v>46111</v>
       </c>
       <c r="G13" s="14"/>
-      <c r="H13" s="14">
-        <f t="shared" ca="1" si="5"/>
-        <v>3</v>
-      </c>
+      <c r="H13" s="14"/>
       <c r="I13" s="31"/>
       <c r="J13" s="31"/>
       <c r="K13" s="31"/>
@@ -3055,7 +3128,7 @@
       <c r="V13" s="31"/>
       <c r="W13" s="31"/>
       <c r="X13" s="31"/>
-      <c r="Y13" s="31"/>
+      <c r="Y13" s="32"/>
       <c r="Z13" s="31"/>
       <c r="AA13" s="31"/>
       <c r="AB13" s="31"/>
@@ -3096,21 +3169,29 @@
       <c r="BK13" s="31"/>
       <c r="BL13" s="31"/>
     </row>
-    <row r="14" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A14" s="46" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C14" s="54"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="73"/>
-      <c r="F14" s="74"/>
+    <row r="14" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="45"/>
+      <c r="B14" s="85" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="86" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="17">
+        <v>1</v>
+      </c>
+      <c r="E14" s="69">
+        <f>E10+1</f>
+        <v>46109</v>
+      </c>
+      <c r="F14" s="69">
+        <f>E14+2</f>
+        <v>46111</v>
+      </c>
       <c r="G14" s="14"/>
-      <c r="H14" s="14" t="str">
+      <c r="H14" s="14">
         <f t="shared" si="5"/>
-        <v/>
+        <v>3</v>
       </c>
       <c r="I14" s="31"/>
       <c r="J14" s="31"/>
@@ -3169,27 +3250,21 @@
       <c r="BK14" s="31"/>
       <c r="BL14" s="31"/>
     </row>
-    <row r="15" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A15" s="46"/>
-      <c r="B15" s="62" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="55"/>
-      <c r="D15" s="20">
-        <v>0.5</v>
-      </c>
-      <c r="E15" s="75">
-        <f ca="1">E13+1</f>
-        <v>46113</v>
-      </c>
-      <c r="F15" s="75">
-        <f ca="1">E15+4</f>
-        <v>46117</v>
-      </c>
+    <row r="15" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="53"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="70"/>
+      <c r="F15" s="71"/>
       <c r="G15" s="14"/>
-      <c r="H15" s="14">
-        <f t="shared" ca="1" si="5"/>
-        <v>5</v>
+      <c r="H15" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v/>
       </c>
       <c r="I15" s="31"/>
       <c r="J15" s="31"/>
@@ -3248,27 +3323,27 @@
       <c r="BK15" s="31"/>
       <c r="BL15" s="31"/>
     </row>
-    <row r="16" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A16" s="45"/>
-      <c r="B16" s="62" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="55"/>
+    <row r="16" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="46"/>
+      <c r="B16" s="87" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="54"/>
       <c r="D16" s="20">
-        <v>0.5</v>
-      </c>
-      <c r="E16" s="75">
-        <f ca="1">E15+2</f>
-        <v>46115</v>
-      </c>
-      <c r="F16" s="75">
-        <f ca="1">E16+5</f>
-        <v>46120</v>
+        <v>0</v>
+      </c>
+      <c r="E16" s="72">
+        <f>E14+1</f>
+        <v>46110</v>
+      </c>
+      <c r="F16" s="72">
+        <f>E16+4</f>
+        <v>46114</v>
       </c>
       <c r="G16" s="14"/>
       <c r="H16" s="14">
-        <f t="shared" ca="1" si="5"/>
-        <v>6</v>
+        <f t="shared" si="5"/>
+        <v>5</v>
       </c>
       <c r="I16" s="31"/>
       <c r="J16" s="31"/>
@@ -3282,8 +3357,8 @@
       <c r="R16" s="31"/>
       <c r="S16" s="31"/>
       <c r="T16" s="31"/>
-      <c r="U16" s="32"/>
-      <c r="V16" s="32"/>
+      <c r="U16" s="31"/>
+      <c r="V16" s="31"/>
       <c r="W16" s="31"/>
       <c r="X16" s="31"/>
       <c r="Y16" s="31"/>
@@ -3327,25 +3402,27 @@
       <c r="BK16" s="31"/>
       <c r="BL16" s="31"/>
     </row>
-    <row r="17" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="17" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="45"/>
-      <c r="B17" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="C17" s="55"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="75">
-        <f ca="1">F16</f>
-        <v>46120</v>
-      </c>
-      <c r="F17" s="75">
-        <f ca="1">E17+3</f>
-        <v>46123</v>
+      <c r="B17" s="87" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="54"/>
+      <c r="D17" s="20">
+        <v>0</v>
+      </c>
+      <c r="E17" s="72">
+        <f>E16+2</f>
+        <v>46112</v>
+      </c>
+      <c r="F17" s="72">
+        <f>E17+5</f>
+        <v>46117</v>
       </c>
       <c r="G17" s="14"/>
       <c r="H17" s="14">
-        <f t="shared" ca="1" si="5"/>
-        <v>4</v>
+        <f t="shared" si="5"/>
+        <v>6</v>
       </c>
       <c r="I17" s="31"/>
       <c r="J17" s="31"/>
@@ -3359,8 +3436,8 @@
       <c r="R17" s="31"/>
       <c r="S17" s="31"/>
       <c r="T17" s="31"/>
-      <c r="U17" s="31"/>
-      <c r="V17" s="31"/>
+      <c r="U17" s="32"/>
+      <c r="V17" s="32"/>
       <c r="W17" s="31"/>
       <c r="X17" s="31"/>
       <c r="Y17" s="31"/>
@@ -3404,25 +3481,29 @@
       <c r="BK17" s="31"/>
       <c r="BL17" s="31"/>
     </row>
-    <row r="18" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="45"/>
-      <c r="B18" s="62" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="55"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="75">
-        <f ca="1">E17</f>
+      <c r="B18" s="87" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="54" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="20">
+        <v>0</v>
+      </c>
+      <c r="E18" s="72">
+        <f>F17</f>
+        <v>46117</v>
+      </c>
+      <c r="F18" s="72">
+        <f>E18+3</f>
         <v>46120</v>
-      </c>
-      <c r="F18" s="75">
-        <f ca="1">E18+2</f>
-        <v>46122</v>
       </c>
       <c r="G18" s="14"/>
       <c r="H18" s="14">
-        <f t="shared" ca="1" si="5"/>
-        <v>3</v>
+        <f t="shared" si="5"/>
+        <v>4</v>
       </c>
       <c r="I18" s="31"/>
       <c r="J18" s="31"/>
@@ -3440,7 +3521,7 @@
       <c r="V18" s="31"/>
       <c r="W18" s="31"/>
       <c r="X18" s="31"/>
-      <c r="Y18" s="32"/>
+      <c r="Y18" s="31"/>
       <c r="Z18" s="31"/>
       <c r="AA18" s="31"/>
       <c r="AB18" s="31"/>
@@ -3481,25 +3562,29 @@
       <c r="BK18" s="31"/>
       <c r="BL18" s="31"/>
     </row>
-    <row r="19" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="45"/>
-      <c r="B19" s="62" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" s="55"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="75">
-        <f ca="1">E18</f>
-        <v>46120</v>
-      </c>
-      <c r="F19" s="75">
-        <f ca="1">E19+3</f>
-        <v>46123</v>
+      <c r="B19" s="87" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="54" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="20">
+        <v>0</v>
+      </c>
+      <c r="E19" s="72">
+        <f>E18</f>
+        <v>46117</v>
+      </c>
+      <c r="F19" s="72">
+        <f>E19+2</f>
+        <v>46119</v>
       </c>
       <c r="G19" s="14"/>
       <c r="H19" s="14">
-        <f t="shared" ca="1" si="5"/>
-        <v>4</v>
+        <f t="shared" si="5"/>
+        <v>3</v>
       </c>
       <c r="I19" s="31"/>
       <c r="J19" s="31"/>
@@ -3517,7 +3602,7 @@
       <c r="V19" s="31"/>
       <c r="W19" s="31"/>
       <c r="X19" s="31"/>
-      <c r="Y19" s="31"/>
+      <c r="Y19" s="32"/>
       <c r="Z19" s="31"/>
       <c r="AA19" s="31"/>
       <c r="AB19" s="31"/>
@@ -3559,20 +3644,28 @@
       <c r="BL19" s="31"/>
     </row>
     <row r="20" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A20" s="45" t="s">
-        <v>11</v>
-      </c>
-      <c r="B20" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="56"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="76"/>
-      <c r="F20" s="77"/>
+      <c r="A20" s="45"/>
+      <c r="B20" s="87" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="54" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="20">
+        <v>0</v>
+      </c>
+      <c r="E20" s="72">
+        <f>E19</f>
+        <v>46117</v>
+      </c>
+      <c r="F20" s="72">
+        <f>E20+3</f>
+        <v>46120</v>
+      </c>
       <c r="G20" s="14"/>
-      <c r="H20" s="14" t="str">
+      <c r="H20" s="14">
         <f t="shared" si="5"/>
-        <v/>
+        <v>4</v>
       </c>
       <c r="I20" s="31"/>
       <c r="J20" s="31"/>
@@ -3632,24 +3725,20 @@
       <c r="BL20" s="31"/>
     </row>
     <row r="21" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A21" s="45"/>
-      <c r="B21" s="63" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" s="57"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="78">
-        <f ca="1">E9+15</f>
-        <v>46123</v>
-      </c>
-      <c r="F21" s="78">
-        <f ca="1">E21+5</f>
-        <v>46128</v>
-      </c>
+      <c r="A21" s="45" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" s="55"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="73"/>
+      <c r="F21" s="74"/>
       <c r="G21" s="14"/>
-      <c r="H21" s="14">
-        <f t="shared" ca="1" si="5"/>
-        <v>6</v>
+      <c r="H21" s="14" t="str">
+        <f t="shared" si="5"/>
+        <v/>
       </c>
       <c r="I21" s="31"/>
       <c r="J21" s="31"/>
@@ -3710,23 +3799,27 @@
     </row>
     <row r="22" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A22" s="45"/>
-      <c r="B22" s="63" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="57"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="78">
-        <f ca="1">F21+1</f>
-        <v>46129</v>
-      </c>
-      <c r="F22" s="78">
-        <f ca="1">E22+4</f>
-        <v>46133</v>
+      <c r="B22" s="60" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="56" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="23">
+        <v>0</v>
+      </c>
+      <c r="E22" s="75">
+        <f ca="1">E9+15</f>
+        <v>46123</v>
+      </c>
+      <c r="F22" s="75">
+        <f ca="1">E22+5</f>
+        <v>46128</v>
       </c>
       <c r="G22" s="14"/>
       <c r="H22" s="14">
         <f t="shared" ca="1" si="5"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I22" s="31"/>
       <c r="J22" s="31"/>
@@ -3787,23 +3880,27 @@
     </row>
     <row r="23" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A23" s="45"/>
-      <c r="B23" s="63" t="s">
-        <v>20</v>
-      </c>
-      <c r="C23" s="57"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="78">
-        <f ca="1">E22+5</f>
-        <v>46134</v>
-      </c>
-      <c r="F23" s="78">
-        <f ca="1">E23+5</f>
-        <v>46139</v>
+      <c r="B23" s="60" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="56" t="s">
+        <v>36</v>
+      </c>
+      <c r="D23" s="23">
+        <v>0</v>
+      </c>
+      <c r="E23" s="75">
+        <f ca="1">F22+1</f>
+        <v>46129</v>
+      </c>
+      <c r="F23" s="75">
+        <f ca="1">E23+4</f>
+        <v>46133</v>
       </c>
       <c r="G23" s="14"/>
       <c r="H23" s="14">
         <f t="shared" ca="1" si="5"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I23" s="31"/>
       <c r="J23" s="31"/>
@@ -3862,25 +3959,29 @@
       <c r="BK23" s="31"/>
       <c r="BL23" s="31"/>
     </row>
-    <row r="24" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="24" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="45"/>
-      <c r="B24" s="63" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24" s="57"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="78">
-        <f ca="1">F23+1</f>
-        <v>46140</v>
-      </c>
-      <c r="F24" s="78">
-        <f ca="1">E24+4</f>
-        <v>46144</v>
+      <c r="B24" s="60" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="56" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="23">
+        <v>0</v>
+      </c>
+      <c r="E24" s="75">
+        <f ca="1">E23+5</f>
+        <v>46134</v>
+      </c>
+      <c r="F24" s="75">
+        <f ca="1">E24+5</f>
+        <v>46139</v>
       </c>
       <c r="G24" s="14"/>
       <c r="H24" s="14">
         <f t="shared" ca="1" si="5"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I24" s="31"/>
       <c r="J24" s="31"/>
@@ -3939,26 +4040,27 @@
       <c r="BK24" s="31"/>
       <c r="BL24" s="31"/>
     </row>
-    <row r="25" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="25" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="45"/>
-      <c r="B25" s="63" t="s">
+      <c r="B25" s="60" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="56" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="57"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="78">
-        <f ca="1">E23</f>
-        <v>46134</v>
-      </c>
-      <c r="F25" s="78">
-        <f ca="1">E25+4</f>
-        <v>46138</v>
+      <c r="D25" s="23">
+        <v>0</v>
+      </c>
+      <c r="E25" s="75">
+        <f ca="1">E24+5</f>
+        <v>46139</v>
+      </c>
+      <c r="F25" s="75">
+        <f ca="1">E25+5</f>
+        <v>46144</v>
       </c>
       <c r="G25" s="14"/>
-      <c r="H25" s="14">
-        <f t="shared" ca="1" si="5"/>
-        <v>5</v>
-      </c>
+      <c r="H25" s="14"/>
       <c r="I25" s="31"/>
       <c r="J25" s="31"/>
       <c r="K25" s="31"/>
@@ -4016,21 +4118,29 @@
       <c r="BK25" s="31"/>
       <c r="BL25" s="31"/>
     </row>
-    <row r="26" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A26" s="45" t="s">
-        <v>11</v>
-      </c>
-      <c r="B26" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="C26" s="58"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="79"/>
-      <c r="F26" s="80"/>
+    <row r="26" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A26" s="45"/>
+      <c r="B26" s="60" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26" s="56" t="s">
+        <v>22</v>
+      </c>
+      <c r="D26" s="23">
+        <v>0</v>
+      </c>
+      <c r="E26" s="75">
+        <f ca="1">F24+1</f>
+        <v>46140</v>
+      </c>
+      <c r="F26" s="75">
+        <f ca="1">E26+4</f>
+        <v>46144</v>
+      </c>
       <c r="G26" s="14"/>
-      <c r="H26" s="14" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="H26" s="14">
+        <f t="shared" ca="1" si="5"/>
+        <v>5</v>
       </c>
       <c r="I26" s="31"/>
       <c r="J26" s="31"/>
@@ -4089,23 +4199,21 @@
       <c r="BK26" s="31"/>
       <c r="BL26" s="31"/>
     </row>
-    <row r="27" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A27" s="45"/>
-      <c r="B27" s="64" t="s">
-        <v>18</v>
-      </c>
-      <c r="C27" s="59"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="81" t="s">
-        <v>33</v>
-      </c>
-      <c r="F27" s="81" t="s">
-        <v>33</v>
-      </c>
+    <row r="27" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A27" s="45" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="C27" s="57"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="76"/>
+      <c r="F27" s="77"/>
       <c r="G27" s="14"/>
-      <c r="H27" s="14" t="e">
+      <c r="H27" s="14" t="str">
         <f t="shared" si="5"/>
-        <v>#VALUE!</v>
+        <v/>
       </c>
       <c r="I27" s="31"/>
       <c r="J27" s="31"/>
@@ -4166,16 +4274,18 @@
     </row>
     <row r="28" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A28" s="45"/>
-      <c r="B28" s="64" t="s">
-        <v>19</v>
-      </c>
-      <c r="C28" s="59"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="81" t="s">
-        <v>33</v>
-      </c>
-      <c r="F28" s="81" t="s">
-        <v>33</v>
+      <c r="B28" s="61" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="58"/>
+      <c r="D28" s="26">
+        <v>0</v>
+      </c>
+      <c r="E28" s="78" t="s">
+        <v>50</v>
+      </c>
+      <c r="F28" s="78" t="s">
+        <v>50</v>
       </c>
       <c r="G28" s="14"/>
       <c r="H28" s="14" t="e">
@@ -4241,16 +4351,18 @@
     </row>
     <row r="29" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A29" s="45"/>
-      <c r="B29" s="64" t="s">
-        <v>20</v>
-      </c>
-      <c r="C29" s="59"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="81" t="s">
-        <v>33</v>
-      </c>
-      <c r="F29" s="81" t="s">
-        <v>33</v>
+      <c r="B29" s="61" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" s="58"/>
+      <c r="D29" s="26">
+        <v>0</v>
+      </c>
+      <c r="E29" s="78" t="s">
+        <v>50</v>
+      </c>
+      <c r="F29" s="78" t="s">
+        <v>50</v>
       </c>
       <c r="G29" s="14"/>
       <c r="H29" s="14" t="e">
@@ -4316,16 +4428,18 @@
     </row>
     <row r="30" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A30" s="45"/>
-      <c r="B30" s="64" t="s">
-        <v>21</v>
-      </c>
-      <c r="C30" s="59"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="81" t="s">
-        <v>33</v>
-      </c>
-      <c r="F30" s="81" t="s">
-        <v>33</v>
+      <c r="B30" s="61" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" s="58"/>
+      <c r="D30" s="26">
+        <v>0</v>
+      </c>
+      <c r="E30" s="78" t="s">
+        <v>50</v>
+      </c>
+      <c r="F30" s="78" t="s">
+        <v>50</v>
       </c>
       <c r="G30" s="14"/>
       <c r="H30" s="14" t="e">
@@ -4391,16 +4505,18 @@
     </row>
     <row r="31" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A31" s="45"/>
-      <c r="B31" s="64" t="s">
-        <v>22</v>
-      </c>
-      <c r="C31" s="59"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="81" t="s">
-        <v>33</v>
-      </c>
-      <c r="F31" s="81" t="s">
-        <v>33</v>
+      <c r="B31" s="61" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" s="58"/>
+      <c r="D31" s="26">
+        <v>0</v>
+      </c>
+      <c r="E31" s="78" t="s">
+        <v>50</v>
+      </c>
+      <c r="F31" s="78" t="s">
+        <v>50</v>
       </c>
       <c r="G31" s="14"/>
       <c r="H31" s="14" t="e">
@@ -4465,18 +4581,24 @@
       <c r="BL31" s="31"/>
     </row>
     <row r="32" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A32" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="B32" s="65"/>
-      <c r="C32" s="60"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="82"/>
-      <c r="F32" s="82"/>
+      <c r="A32" s="45"/>
+      <c r="B32" s="61" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="58"/>
+      <c r="D32" s="26">
+        <v>0</v>
+      </c>
+      <c r="E32" s="78" t="s">
+        <v>50</v>
+      </c>
+      <c r="F32" s="78" t="s">
+        <v>50</v>
+      </c>
       <c r="G32" s="14"/>
-      <c r="H32" s="14" t="str">
+      <c r="H32" s="14" t="e">
         <f t="shared" si="5"/>
-        <v/>
+        <v>#VALUE!</v>
       </c>
       <c r="I32" s="31"/>
       <c r="J32" s="31"/>
@@ -4536,103 +4658,174 @@
       <c r="BL32" s="31"/>
     </row>
     <row r="33" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A33" s="46" t="s">
-        <v>13</v>
-      </c>
-      <c r="B33" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="C33" s="28"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="83"/>
-      <c r="F33" s="84"/>
-      <c r="G33" s="30"/>
-      <c r="H33" s="30" t="str">
+      <c r="A33" s="45" t="s">
+        <v>55</v>
+      </c>
+      <c r="B33" s="62"/>
+      <c r="C33" s="59"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="79"/>
+      <c r="F33" s="79"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="I33" s="33"/>
-      <c r="J33" s="33"/>
-      <c r="K33" s="33"/>
-      <c r="L33" s="33"/>
-      <c r="M33" s="33"/>
-      <c r="N33" s="33"/>
-      <c r="O33" s="33"/>
-      <c r="P33" s="33"/>
-      <c r="Q33" s="33"/>
-      <c r="R33" s="33"/>
-      <c r="S33" s="33"/>
-      <c r="T33" s="33"/>
-      <c r="U33" s="33"/>
-      <c r="V33" s="33"/>
-      <c r="W33" s="33"/>
-      <c r="X33" s="33"/>
-      <c r="Y33" s="33"/>
-      <c r="Z33" s="33"/>
-      <c r="AA33" s="33"/>
-      <c r="AB33" s="33"/>
-      <c r="AC33" s="33"/>
-      <c r="AD33" s="33"/>
-      <c r="AE33" s="33"/>
-      <c r="AF33" s="33"/>
-      <c r="AG33" s="33"/>
-      <c r="AH33" s="33"/>
-      <c r="AI33" s="33"/>
-      <c r="AJ33" s="33"/>
-      <c r="AK33" s="33"/>
-      <c r="AL33" s="33"/>
-      <c r="AM33" s="33"/>
-      <c r="AN33" s="33"/>
-      <c r="AO33" s="33"/>
-      <c r="AP33" s="33"/>
-      <c r="AQ33" s="33"/>
-      <c r="AR33" s="33"/>
-      <c r="AS33" s="33"/>
-      <c r="AT33" s="33"/>
-      <c r="AU33" s="33"/>
-      <c r="AV33" s="33"/>
-      <c r="AW33" s="33"/>
-      <c r="AX33" s="33"/>
-      <c r="AY33" s="33"/>
-      <c r="AZ33" s="33"/>
-      <c r="BA33" s="33"/>
-      <c r="BB33" s="33"/>
-      <c r="BC33" s="33"/>
-      <c r="BD33" s="33"/>
-      <c r="BE33" s="33"/>
-      <c r="BF33" s="33"/>
-      <c r="BG33" s="33"/>
-      <c r="BH33" s="33"/>
-      <c r="BI33" s="33"/>
-      <c r="BJ33" s="33"/>
-      <c r="BK33" s="33"/>
-      <c r="BL33" s="33"/>
+      <c r="I33" s="31"/>
+      <c r="J33" s="31"/>
+      <c r="K33" s="31"/>
+      <c r="L33" s="31"/>
+      <c r="M33" s="31"/>
+      <c r="N33" s="31"/>
+      <c r="O33" s="31"/>
+      <c r="P33" s="31"/>
+      <c r="Q33" s="31"/>
+      <c r="R33" s="31"/>
+      <c r="S33" s="31"/>
+      <c r="T33" s="31"/>
+      <c r="U33" s="31"/>
+      <c r="V33" s="31"/>
+      <c r="W33" s="31"/>
+      <c r="X33" s="31"/>
+      <c r="Y33" s="31"/>
+      <c r="Z33" s="31"/>
+      <c r="AA33" s="31"/>
+      <c r="AB33" s="31"/>
+      <c r="AC33" s="31"/>
+      <c r="AD33" s="31"/>
+      <c r="AE33" s="31"/>
+      <c r="AF33" s="31"/>
+      <c r="AG33" s="31"/>
+      <c r="AH33" s="31"/>
+      <c r="AI33" s="31"/>
+      <c r="AJ33" s="31"/>
+      <c r="AK33" s="31"/>
+      <c r="AL33" s="31"/>
+      <c r="AM33" s="31"/>
+      <c r="AN33" s="31"/>
+      <c r="AO33" s="31"/>
+      <c r="AP33" s="31"/>
+      <c r="AQ33" s="31"/>
+      <c r="AR33" s="31"/>
+      <c r="AS33" s="31"/>
+      <c r="AT33" s="31"/>
+      <c r="AU33" s="31"/>
+      <c r="AV33" s="31"/>
+      <c r="AW33" s="31"/>
+      <c r="AX33" s="31"/>
+      <c r="AY33" s="31"/>
+      <c r="AZ33" s="31"/>
+      <c r="BA33" s="31"/>
+      <c r="BB33" s="31"/>
+      <c r="BC33" s="31"/>
+      <c r="BD33" s="31"/>
+      <c r="BE33" s="31"/>
+      <c r="BF33" s="31"/>
+      <c r="BG33" s="31"/>
+      <c r="BH33" s="31"/>
+      <c r="BI33" s="31"/>
+      <c r="BJ33" s="31"/>
+      <c r="BK33" s="31"/>
+      <c r="BL33" s="31"/>
     </row>
-    <row r="34" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="G34" s="6"/>
+    <row r="34" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A34" s="46" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" s="27" t="s">
+        <v>57</v>
+      </c>
+      <c r="C34" s="28"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="80"/>
+      <c r="F34" s="81"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="30" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="I34" s="33"/>
+      <c r="J34" s="33"/>
+      <c r="K34" s="33"/>
+      <c r="L34" s="33"/>
+      <c r="M34" s="33"/>
+      <c r="N34" s="33"/>
+      <c r="O34" s="33"/>
+      <c r="P34" s="33"/>
+      <c r="Q34" s="33"/>
+      <c r="R34" s="33"/>
+      <c r="S34" s="33"/>
+      <c r="T34" s="33"/>
+      <c r="U34" s="33"/>
+      <c r="V34" s="33"/>
+      <c r="W34" s="33"/>
+      <c r="X34" s="33"/>
+      <c r="Y34" s="33"/>
+      <c r="Z34" s="33"/>
+      <c r="AA34" s="33"/>
+      <c r="AB34" s="33"/>
+      <c r="AC34" s="33"/>
+      <c r="AD34" s="33"/>
+      <c r="AE34" s="33"/>
+      <c r="AF34" s="33"/>
+      <c r="AG34" s="33"/>
+      <c r="AH34" s="33"/>
+      <c r="AI34" s="33"/>
+      <c r="AJ34" s="33"/>
+      <c r="AK34" s="33"/>
+      <c r="AL34" s="33"/>
+      <c r="AM34" s="33"/>
+      <c r="AN34" s="33"/>
+      <c r="AO34" s="33"/>
+      <c r="AP34" s="33"/>
+      <c r="AQ34" s="33"/>
+      <c r="AR34" s="33"/>
+      <c r="AS34" s="33"/>
+      <c r="AT34" s="33"/>
+      <c r="AU34" s="33"/>
+      <c r="AV34" s="33"/>
+      <c r="AW34" s="33"/>
+      <c r="AX34" s="33"/>
+      <c r="AY34" s="33"/>
+      <c r="AZ34" s="33"/>
+      <c r="BA34" s="33"/>
+      <c r="BB34" s="33"/>
+      <c r="BC34" s="33"/>
+      <c r="BD34" s="33"/>
+      <c r="BE34" s="33"/>
+      <c r="BF34" s="33"/>
+      <c r="BG34" s="33"/>
+      <c r="BH34" s="33"/>
+      <c r="BI34" s="33"/>
+      <c r="BJ34" s="33"/>
+      <c r="BK34" s="33"/>
+      <c r="BL34" s="33"/>
     </row>
     <row r="35" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C35" s="11"/>
-      <c r="F35" s="47"/>
+      <c r="G35" s="6"/>
     </row>
     <row r="36" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C36" s="12"/>
+      <c r="C36" s="11"/>
+      <c r="F36" s="47"/>
+    </row>
+    <row r="37" spans="1:64" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C37" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="AK4:AQ4"/>
+    <mergeCell ref="AR4:AX4"/>
+    <mergeCell ref="AY4:BE4"/>
     <mergeCell ref="BF4:BL4"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="I4:O4"/>
     <mergeCell ref="P4:V4"/>
     <mergeCell ref="W4:AC4"/>
     <mergeCell ref="AD4:AJ4"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="AK4:AQ4"/>
-    <mergeCell ref="AR4:AX4"/>
-    <mergeCell ref="AY4:BE4"/>
   </mergeCells>
-  <conditionalFormatting sqref="D7:D33">
+  <conditionalFormatting sqref="D7:D34">
     <cfRule type="dataBar" priority="14">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -4646,17 +4839,24 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:BL33">
-    <cfRule type="expression" dxfId="2" priority="33">
+  <conditionalFormatting sqref="I5:BL8 I9:R9 T9:BL9 I10:BL34">
+    <cfRule type="expression" dxfId="3" priority="33">
       <formula>AND(TODAY()&gt;=I$5,TODAY()&lt;J$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I7:BL33">
+  <conditionalFormatting sqref="I7:BL8 I9:L9 N9:R9 T9:BL9 I10:BL34">
+    <cfRule type="expression" dxfId="2" priority="28" stopIfTrue="1">
+      <formula>AND(task_end&gt;=I$5,task_start&lt;J$5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I7:BL8 I9:R9 T9:BL9 I10:BL34">
     <cfRule type="expression" dxfId="1" priority="27">
       <formula>AND(task_start&lt;=I$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="28" stopIfTrue="1">
-      <formula>AND(task_end&gt;=I$5,task_start&lt;J$5)</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M9">
+    <cfRule type="expression" dxfId="0" priority="39" stopIfTrue="1">
+      <formula>AND(task_end&gt;=M$5,task_start&lt;N$5)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -4664,18 +4864,14 @@
       <formula1>1</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="I2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="I1" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-  </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.5" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="60" fitToHeight="0" orientation="landscape" r:id="rId3"/>
+  <pageSetup paperSize="9" scale="60" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter differentFirst="1" scaleWithDoc="0">
     <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <ignoredErrors>
-    <ignoredError sqref="F18 F22:F23 E23" formula="1"/>
+    <ignoredError sqref="F19 F23:F24 E24" formula="1"/>
   </ignoredErrors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -4693,7 +4889,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D7:D33</xm:sqref>
+          <xm:sqref>D7:D34</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4713,79 +4909,79 @@
     <row r="1" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="2" spans="1:2" s="37" customFormat="1" ht="15.75" x14ac:dyDescent="0.45">
       <c r="A2" s="36" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="B2" s="36"/>
     </row>
     <row r="3" spans="1:2" s="41" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="69" t="s">
-        <v>37</v>
+      <c r="A3" s="66" t="s">
+        <v>59</v>
       </c>
       <c r="B3" s="42"/>
     </row>
     <row r="4" spans="1:2" s="38" customFormat="1" ht="25.5" x14ac:dyDescent="0.75">
       <c r="A4" s="39" t="s">
-        <v>38</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="74.099999999999994" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="40" t="s">
-        <v>39</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="39" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="35" customFormat="1" ht="204.95" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="44" t="s">
-        <v>41</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="38" customFormat="1" ht="25.5" x14ac:dyDescent="0.75">
       <c r="A8" s="39" t="s">
-        <v>42</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="40" t="s">
-        <v>43</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:2" s="35" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="43" t="s">
-        <v>44</v>
+        <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="38" customFormat="1" ht="25.5" x14ac:dyDescent="0.75">
       <c r="A11" s="39" t="s">
-        <v>45</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="40" t="s">
-        <v>46</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:2" s="35" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="43" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:2" s="38" customFormat="1" ht="25.5" x14ac:dyDescent="0.75">
       <c r="A14" s="39" t="s">
-        <v>48</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="40" t="s">
-        <v>49</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="40" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -4802,58 +4998,33 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="24" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2d714a3296df14eba7a100bb665443ca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="49549bf45bfbbfb6cffed527380e77e1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
-    <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
-    <xsd:import namespace="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <xsd:import namespace="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <xsd:import namespace="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100A8A2461AC630654B81BDF11CF52C49F7" ma:contentTypeVersion="9" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="a9f765ae97f268f9db914e6a1a6a0bc8">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="38fcf7b7-71b2-4d8e-9cff-ecdc863721c8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4cedfb0b4d812b3ae33e4a46bb7bcf26" ns3:_="">
+    <xsd:import namespace="38fcf7b7-71b2-4d8e-9cff-ecdc863721c8"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element name="documentManagement">
             <xsd:complexType>
               <xsd:all>
-                <xsd:element ref="ns2:Status" minOccurs="0"/>
-                <xsd:element ref="ns2:Image" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoTags" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceAutoKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceKeyPoints" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyProperties" minOccurs="0"/>
-                <xsd:element ref="ns1:_ip_UnifiedCompliancePolicyUIAction" minOccurs="0"/>
-                <xsd:element ref="ns4:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:ImageTagsTaxHTField" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:Background" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns3:_activity" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSystemTags" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceOCR" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -4861,153 +5032,55 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="http://schemas.microsoft.com/sharepoint/v3" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="38fcf7b7-71b2-4d8e-9cff-ecdc863721c8" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="_ip_UnifiedCompliancePolicyProperties" ma:index="20" nillable="true" ma:displayName="Unified Compliance Policy Properties" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyProperties" ma:readOnly="false">
+    <xsd:element name="MediaServiceDateTaken" ma:index="8" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="_activity" ma:index="9" nillable="true" ma:displayName="_activity" ma:hidden="true" ma:internalName="_activity">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="_ip_UnifiedCompliancePolicyUIAction" ma:index="21" nillable="true" ma:displayName="Unified Compliance Policy UI Action" ma:hidden="true" ma:internalName="_ip_UnifiedCompliancePolicyUIAction" ma:readOnly="false">
+    <xsd:element name="MediaServiceMetadata" ma:index="10" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="12" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSystemTags" ma:index="13" nillable="true" ma:displayName="MediaServiceSystemTags" ma:hidden="true" ma:internalName="MediaServiceSystemTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="14" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="Status" ma:index="2" nillable="true" ma:displayName="Status" ma:default="Not started" ma:format="Dropdown" ma:internalName="Status" ma:readOnly="false">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Choice">
-          <xsd:enumeration value="Not started"/>
-          <xsd:enumeration value="In Progress"/>
-          <xsd:enumeration value="Completed"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Image" ma:index="3" nillable="true" ma:displayName="Image" ma:format="Image" ma:internalName="Image" ma:readOnly="false">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:URL">
-            <xsd:sequence>
-              <xsd:element name="Url" type="dms:ValidUrl" minOccurs="0" nillable="true"/>
-              <xsd:element name="Description" type="xsd:string" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="10" nillable="true" ma:displayName="MediaServiceOCR" ma:hidden="true" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoTags" ma:index="11" nillable="true" ma:displayName="MediaServiceAutoTags" ma:hidden="true" ma:internalName="MediaServiceAutoTags" ma:readOnly="true">
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="12" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
       <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
       </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceAutoKeyPoints" ma:index="16" nillable="true" ma:displayName="MediaServiceAutoKeyPoints" ma:hidden="true" ma:internalName="MediaServiceAutoKeyPoints" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceKeyPoints" ma:index="17" nillable="true" ma:displayName="KeyPoints" ma:hidden="true" ma:internalName="MediaServiceKeyPoints" ma:readOnly="false">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="18" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="ImageTagsTaxHTField" ma:index="25" nillable="true" ma:taxonomy="true" ma:internalName="ImageTagsTaxHTField" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="e385fb40-52d4-4fae-9c5b-3e8ff8a5878e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="26" nillable="true" ma:displayName="Location" ma:hidden="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="27" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Background" ma:index="28" nillable="true" ma:displayName="Background" ma:default="0" ma:format="Dropdown" ma:internalName="Background">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Boolean"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="16c05727-aa75-4e4a-9b5f-8a80a1165891" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="14" nillable="true" ma:displayName="Shared With" ma:hidden="true" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="15" nillable="true" ma:displayName="Shared With Details" ma:hidden="true" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="230e9df3-be65-4c73-a93b-d1236ebd677e" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="23" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3f6bfcbc-3db3-4ae6-bd76-326f0798ad28}" ma:internalName="TaxCatchAll" ma:readOnly="false" ma:showField="CatchAllData" ma:web="16c05727-aa75-4e4a-9b5f-8a80a1165891">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -5019,8 +5092,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="1" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Inhaltstyp"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titel"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -5110,37 +5183,29 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="38fcf7b7-71b2-4d8e-9cff-ecdc863721c8" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F80F839-78EF-4FF4-A673-3CC84279C232}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{63C14AF3-3041-4092-A567-C704F7642EEF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
     <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="16c05727-aa75-4e4a-9b5f-8a80a1165891"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="38fcf7b7-71b2-4d8e-9cff-ecdc863721c8"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
@@ -5152,9 +5217,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4A34E49-7289-4AEA-9593-4F55E04ADB10}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AC3AD2E1-977A-4D4F-8EE8-D64B5FFADF75}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="38fcf7b7-71b2-4d8e-9cff-ecdc863721c8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>